<commit_message>
feat(fisica): integrato grafico a dispersione nativo automatico nei file Excel scheda_laboratorio e scheda_velocita
</commit_message>
<xml_diff>
--- a/public/fisica/archimede/seconda-elettronica/scheda_laboratorio_A4.xlsx
+++ b/public/fisica/archimede/seconda-elettronica/scheda_laboratorio_A4.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="22">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,7 +83,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00000000"/>
+      <color rgb="001E3A8A"/>
       <sz val="9"/>
     </font>
     <font>
@@ -111,31 +111,14 @@
     </font>
     <font>
       <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="0015803D"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00475569"/>
-      <sz val="7.5"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
       <color rgb="001E293B"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="0015803D"/>
-      <sz val="6.5"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="001E293B"/>
-      <sz val="8"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -148,6 +131,11 @@
       <b val="1"/>
       <color rgb="000F172A"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00475569"/>
+      <sz val="7.5"/>
     </font>
   </fonts>
   <fills count="11">
@@ -203,7 +191,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -239,181 +227,11 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="000F172A"/>
-      </left>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="001E3A8A"/>
-      </right>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="000F172A"/>
-      </left>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="hair">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="hair">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="001E3A8A"/>
-      </right>
-      <top style="hair">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="000F172A"/>
-      </left>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="hair">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="000F172A"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="hair">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="000F172A"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="hair">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="001E3A8A"/>
-      </right>
-      <top style="hair">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="000F172A"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="hair">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="001E3A8A"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -425,9 +243,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="bottom"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -440,22 +255,6 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -465,9 +264,6 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -482,27 +278,28 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -577,6 +374,158 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="13"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Grafico Spazio-Tempo s(t)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <scatterChart>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Scheda Esperimento'!D6</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="25400">
+              <a:solidFill>
+                <a:srgbClr val="1E3A8A"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="38BDF8"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="1E3A8A"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'Scheda Esperimento'!$C$7:$C$15</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Scheda Esperimento'!$D$7:$D$15</f>
+            </numRef>
+          </yVal>
+        </ser>
+        <axId val="10"/>
+        <axId val="20"/>
+      </scatterChart>
+      <valAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tempo t [s]</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="20"/>
+      </valAx>
+      <valAx>
+        <axId val="20"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Spazio s [m]</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3744000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -876,11 +825,11 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
@@ -888,7 +837,7 @@
     <row r="1" ht="16" customHeight="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>LABORATORIO DI FISICA SPERIMENTALE — I.T.I.S.</t>
+          <t>ISS ARCHIMEDE — LABORATORIO DI FISICA SPERIMENTALE — 2ª ELETTRONICA</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
@@ -908,14 +857,14 @@
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>2ª _________</t>
+          <t>2ª Elettronica</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>IL GRAFICO SPAZIO-TEMPO NEL MOTO RETTILINEO</t>
+          <t>LABORATORIO 1: IL GRAFICO SPAZIO-TEMPO NEL MOTO RETTILINEO</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -935,14 +884,14 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>___ / ___ / 202...</t>
+          <t>10 / 10 / 2026</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Esperienza con rotaia e carrello: studio del moto rettilineo con andata e ritorno</t>
+          <t>Esperienza con rotaia e carrello: studio del moto rettilineo con andata e ritorno (punta 2,30 m)</t>
         </is>
       </c>
     </row>
@@ -955,7 +904,7 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>2. GRAFICO SPAZIO-TEMPO (da tracciare a mano e su Excel)</t>
+          <t>2. GRAFICO SPAZIO-TEMPO s(t) — AUTOMATICO IN TEMPO REALE</t>
         </is>
       </c>
     </row>
@@ -980,351 +929,265 @@
           <t>Note / Evento</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>▲ s [m]</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="17" customHeight="1">
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>Andata</t>
         </is>
       </c>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12" t="n">
+      <c r="C7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="D7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Partenza (t0)</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
-        <is>
-          <t>2,30 —</t>
-        </is>
-      </c>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="17" t="inlineStr">
-        <is>
-          <t>Punta massima a 2,30 m • Griglia (t, s)</t>
-        </is>
-      </c>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="19" t="n"/>
     </row>
     <row r="8" ht="17" customHeight="1">
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Andata</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="12" t="n">
+      <c r="C8" s="10" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="D8" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Traguardo 1</t>
         </is>
       </c>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="21" t="n"/>
-      <c r="I8" s="21" t="n"/>
-      <c r="J8" s="21" t="n"/>
-      <c r="K8" s="21" t="n"/>
-      <c r="L8" s="22" t="n"/>
     </row>
     <row r="9" ht="17" customHeight="1">
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Andata</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="12" t="n">
+      <c r="C9" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Traguardo 2</t>
         </is>
       </c>
-      <c r="F9" s="23" t="inlineStr">
-        <is>
-          <t>2,00 —</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="n"/>
-      <c r="H9" s="21" t="n"/>
-      <c r="I9" s="21" t="n"/>
-      <c r="J9" s="21" t="n"/>
-      <c r="K9" s="21" t="n"/>
-      <c r="L9" s="22" t="n"/>
     </row>
     <row r="10" ht="17" customHeight="1">
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Andata</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="12" t="n">
+      <c r="C10" s="10" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D10" s="11" t="n">
         <v>1.5</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>Traguardo 3 (andata)</t>
         </is>
       </c>
-      <c r="G10" s="20" t="n"/>
-      <c r="H10" s="21" t="n"/>
-      <c r="I10" s="21" t="n"/>
-      <c r="J10" s="21" t="n"/>
-      <c r="K10" s="21" t="n"/>
-      <c r="L10" s="22" t="n"/>
     </row>
     <row r="11" ht="17" customHeight="1">
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Punta</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="25" t="n">
+      <c r="C11" s="10" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="D11" s="14" t="n">
         <v>2.3</v>
       </c>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Inversione (punta)</t>
         </is>
       </c>
-      <c r="F11" s="27" t="inlineStr">
-        <is>
-          <t>1,50 —</t>
-        </is>
-      </c>
-      <c r="G11" s="20" t="n"/>
-      <c r="H11" s="21" t="n"/>
-      <c r="I11" s="21" t="n"/>
-      <c r="J11" s="21" t="n"/>
-      <c r="K11" s="21" t="n"/>
-      <c r="L11" s="22" t="n"/>
     </row>
     <row r="12" ht="17" customHeight="1">
-      <c r="B12" s="28" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n"/>
-      <c r="D12" s="29" t="n">
+      <c r="C12" s="10" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D12" s="17" t="n">
         <v>1.5</v>
       </c>
-      <c r="E12" s="30" t="inlineStr">
+      <c r="E12" s="18" t="inlineStr">
         <is>
           <t>Traguardo 3 (ritorno)</t>
         </is>
       </c>
-      <c r="G12" s="20" t="n"/>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="21" t="n"/>
-      <c r="L12" s="22" t="n"/>
     </row>
     <row r="13" ht="17" customHeight="1">
-      <c r="B13" s="28" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="29" t="n">
+      <c r="C13" s="10" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="D13" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="30" t="inlineStr">
+      <c r="E13" s="18" t="inlineStr">
         <is>
           <t>Traguardo 2 (ritorno)</t>
         </is>
       </c>
-      <c r="F13" s="27" t="inlineStr">
-        <is>
-          <t>1,00 —</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="n"/>
-      <c r="H13" s="21" t="n"/>
-      <c r="I13" s="21" t="n"/>
-      <c r="J13" s="21" t="n"/>
-      <c r="K13" s="21" t="n"/>
-      <c r="L13" s="22" t="n"/>
     </row>
     <row r="14" ht="17" customHeight="1">
-      <c r="B14" s="28" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C14" s="11" t="n"/>
-      <c r="D14" s="29" t="n">
+      <c r="C14" s="10" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="D14" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="E14" s="30" t="inlineStr">
+      <c r="E14" s="18" t="inlineStr">
         <is>
           <t>Traguardo 1 (ritorno)</t>
         </is>
       </c>
-      <c r="G14" s="20" t="n"/>
-      <c r="H14" s="21" t="n"/>
-      <c r="I14" s="21" t="n"/>
-      <c r="J14" s="21" t="n"/>
-      <c r="K14" s="21" t="n"/>
-      <c r="L14" s="22" t="n"/>
     </row>
     <row r="15" ht="17" customHeight="1">
-      <c r="B15" s="28" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="29" t="n">
+      <c r="C15" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="30" t="inlineStr">
+      <c r="E15" s="18" t="inlineStr">
         <is>
           <t>Rientro al punto iniziale</t>
         </is>
       </c>
-      <c r="F15" s="27" t="inlineStr">
-        <is>
-          <t>0,50 —</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="n"/>
-      <c r="H15" s="21" t="n"/>
-      <c r="I15" s="21" t="n"/>
-      <c r="J15" s="21" t="n"/>
-      <c r="K15" s="21" t="n"/>
-      <c r="L15" s="22" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="B16" s="31" t="inlineStr">
-        <is>
-          <t>📐 ISTRUZIONI: Segna i punti (t, s) sulla griglia a destra (punta a 2,30 m) e uniscili.</t>
-        </is>
-      </c>
-      <c r="C16" s="32" t="n"/>
-      <c r="D16" s="32" t="n"/>
-      <c r="E16" s="32" t="n"/>
-      <c r="G16" s="20" t="n"/>
-      <c r="H16" s="21" t="n"/>
-      <c r="I16" s="21" t="n"/>
-      <c r="J16" s="21" t="n"/>
-      <c r="K16" s="21" t="n"/>
-      <c r="L16" s="22" t="n"/>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>✨ GRAFICO AUTOMATICO: Modifica i tempi nella colonna C, il grafico a destra si aggiorna da solo!</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="n"/>
+      <c r="D16" s="20" t="n"/>
+      <c r="E16" s="20" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>Su Excel: Inserisci le due colonne (Tempo, Spazio), crea Grafico a Dispersione (linee rette).</t>
-        </is>
-      </c>
-      <c r="C17" s="32" t="n"/>
-      <c r="D17" s="32" t="n"/>
-      <c r="E17" s="32" t="n"/>
-      <c r="F17" s="27" t="inlineStr">
-        <is>
-          <t>0,00 —</t>
-        </is>
-      </c>
-      <c r="G17" s="34" t="n"/>
-      <c r="H17" s="35" t="n"/>
-      <c r="I17" s="35" t="n"/>
-      <c r="J17" s="35" t="n"/>
-      <c r="K17" s="35" t="n"/>
-      <c r="L17" s="36" t="n"/>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Punta di inversione a 2,30 m • Il moto passa due volte per s = 1,50 m (andata e ritorno).</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="n"/>
+      <c r="D17" s="20" t="n"/>
+      <c r="E17" s="20" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="B18" s="37" t="inlineStr">
-        <is>
-          <t>Strumenti: Rotaia a cuscino d'aria con carrello e cronometro digitale.</t>
-        </is>
-      </c>
-      <c r="C18" s="32" t="n"/>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="32" t="n"/>
-      <c r="I18" s="38" t="inlineStr">
-        <is>
-          <t>TEMPO t (secondi, s) ►</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="17" customHeight="1">
-      <c r="B19" s="39" t="inlineStr">
-        <is>
-          <t>1. Pendenza Andata: v_andata = Δs / Δt = (2,30 m - 0,00 m) / (t_punta - t_0) = __________________ m/s</t>
-        </is>
-      </c>
-      <c r="J19" s="40" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Strumenti: Rotaia graduata con carrello virtuale e cronometro digitale.</t>
+        </is>
+      </c>
+      <c r="C18" s="20" t="n"/>
+      <c r="D18" s="20" t="n"/>
+      <c r="E18" s="20" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Pendenza Andata: v_andata = (2,30 m - 0,00 m)/(t_punta - t_0)</t>
+        </is>
+      </c>
+      <c r="E19" s="24">
+        <f>(D11-D7)/(C11-C7)</f>
+        <v/>
+      </c>
+      <c r="J19" s="25" t="inlineStr">
         <is>
           <t>VALUTAZIONE DOCENTE</t>
         </is>
       </c>
-      <c r="K19" s="32" t="n"/>
-      <c r="L19" s="32" t="n"/>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="B20" s="39" t="inlineStr">
-        <is>
-          <t>2. Pendenza Ritorno: v_ritorno = Δs / Δt = (0,00 m - 2,30 m) / (t_fine - t_punta) = __________________ m/s</t>
-        </is>
-      </c>
-      <c r="J20" s="41" t="inlineStr">
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="20" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Pendenza Ritorno: v_ritorno = (0,00 m - 2,30 m)/(t_fine - t_punta)</t>
+        </is>
+      </c>
+      <c r="E20" s="26">
+        <f>(D15-D11)/(C15-C11)</f>
+        <v/>
+      </c>
+      <c r="J20" s="27" t="inlineStr">
         <is>
           <t>Voto: ______ / 10</t>
         </is>
       </c>
-      <c r="K20" s="32" t="n"/>
-      <c r="L20" s="42" t="inlineStr">
+      <c r="K20" s="20" t="n"/>
+      <c r="L20" s="28" t="inlineStr">
         <is>
           <t>Firma: ________</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="B21" s="39" t="inlineStr">
-        <is>
-          <t>3. Analisi: Cosa rappresenta la punta a 2,30 m? Perché il grafico passa due volte per s = 1,50 m? ____________________________</t>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>Nota: La pendenza di andata è positiva (+), quella di ritorno è negativa (-) perché il verso è opposto.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="14">
     <mergeCell ref="H1:J1"/>
-    <mergeCell ref="J7:L7"/>
     <mergeCell ref="B17:E17"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="G5:L5"/>
     <mergeCell ref="J20:K20"/>
-    <mergeCell ref="G5:L5"/>
-    <mergeCell ref="I18:L18"/>
-    <mergeCell ref="B21:H21"/>
     <mergeCell ref="J19:L19"/>
+    <mergeCell ref="B21:E21"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B2:E2"/>
     <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B20:H20"/>
+    <mergeCell ref="B20:D20"/>
   </mergeCells>
-  <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(fisica): rimosso PDF statico, svuotati input Excel con formule auto e aggiunto pulsante Best-Fit MRU
</commit_message>
<xml_diff>
--- a/public/fisica/archimede/seconda-elettronica/scheda_laboratorio_A4.xlsx
+++ b/public/fisica/archimede/seconda-elettronica/scheda_laboratorio_A4.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,7 +83,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="001E3A8A"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
@@ -113,6 +113,12 @@
       <name val="Segoe UI"/>
       <color rgb="001E293B"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Segoe UI"/>
@@ -284,19 +290,19 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="2" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="17" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -438,6 +444,7 @@
               <f>'Scheda Esperimento'!$D$7:$D$15</f>
             </numRef>
           </yVal>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="20"/>
@@ -825,13 +832,13 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="2" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="3" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="16" customHeight="1">
@@ -884,7 +891,7 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>10 / 10 / 2026</t>
+          <t>___ / ___ / 202...</t>
         </is>
       </c>
     </row>
@@ -899,7 +906,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1. TABELLA DEI DATI SPERIMENTALI</t>
+          <t>1. TABELLA DEI DATI SPERIMENTALI (DA COMPILARE)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -954,9 +961,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
-        <v>1.25</v>
-      </c>
+      <c r="C8" s="10" t="n"/>
       <c r="D8" s="11" t="n">
         <v>0.5</v>
       </c>
@@ -972,9 +977,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
-        <v>2.5</v>
-      </c>
+      <c r="C9" s="10" t="n"/>
       <c r="D9" s="11" t="n">
         <v>1</v>
       </c>
@@ -990,9 +993,7 @@
           <t>Andata</t>
         </is>
       </c>
-      <c r="C10" s="10" t="n">
-        <v>3.8</v>
-      </c>
+      <c r="C10" s="10" t="n"/>
       <c r="D10" s="11" t="n">
         <v>1.5</v>
       </c>
@@ -1008,9 +1009,7 @@
           <t>Punta</t>
         </is>
       </c>
-      <c r="C11" s="10" t="n">
-        <v>5.5</v>
-      </c>
+      <c r="C11" s="10" t="n"/>
       <c r="D11" s="14" t="n">
         <v>2.3</v>
       </c>
@@ -1026,9 +1025,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n">
-        <v>7.2</v>
-      </c>
+      <c r="C12" s="10" t="n"/>
       <c r="D12" s="17" t="n">
         <v>1.5</v>
       </c>
@@ -1044,9 +1041,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C13" s="10" t="n">
-        <v>8.5</v>
-      </c>
+      <c r="C13" s="10" t="n"/>
       <c r="D13" s="17" t="n">
         <v>1</v>
       </c>
@@ -1062,9 +1057,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
-        <v>9.75</v>
-      </c>
+      <c r="C14" s="10" t="n"/>
       <c r="D14" s="17" t="n">
         <v>0.5</v>
       </c>
@@ -1080,9 +1073,7 @@
           <t>Ritorno</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
-        <v>11</v>
-      </c>
+      <c r="C15" s="10" t="n"/>
       <c r="D15" s="17" t="n">
         <v>0</v>
       </c>
@@ -1095,7 +1086,7 @@
     <row r="16" ht="16" customHeight="1">
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>✨ GRAFICO AUTOMATICO: Modifica i tempi nella colonna C, il grafico a destra si aggiorna da solo!</t>
+          <t>✨ GRAFICO AUTOMATICO: Inserisci i tuoi tempi nella colonna C, il grafico si traccia da solo!</t>
         </is>
       </c>
       <c r="C16" s="20" t="n"/>
@@ -1105,7 +1096,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>Punta di inversione a 2,30 m • Il moto passa due volte per s = 1,50 m (andata e ritorno).</t>
+          <t>Punta di inversione a 2,30 m • Il carrello passa due volte per s = 1,50 m (andata e ritorno).</t>
         </is>
       </c>
       <c r="C17" s="20" t="n"/>
@@ -1122,14 +1113,14 @@
       <c r="D18" s="20" t="n"/>
       <c r="E18" s="20" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1">
+    <row r="19" ht="17" customHeight="1">
       <c r="B19" s="23" t="inlineStr">
         <is>
           <t>Pendenza Andata: v_andata = (2,30 m - 0,00 m)/(t_punta - t_0)</t>
         </is>
       </c>
       <c r="E19" s="24">
-        <f>(D11-D7)/(C11-C7)</f>
+        <f>IF(AND(ISNUMBER(C11), ISNUMBER(C7), C11&gt;C7), ROUND((D11-D7)/(C11-C7), 2), "")</f>
         <v/>
       </c>
       <c r="J19" s="25" t="inlineStr">
@@ -1140,14 +1131,14 @@
       <c r="K19" s="20" t="n"/>
       <c r="L19" s="20" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20" ht="17" customHeight="1">
       <c r="B20" s="23" t="inlineStr">
         <is>
           <t>Pendenza Ritorno: v_ritorno = (0,00 m - 2,30 m)/(t_fine - t_punta)</t>
         </is>
       </c>
       <c r="E20" s="26">
-        <f>(D15-D11)/(C15-C11)</f>
+        <f>IF(AND(ISNUMBER(C15), ISNUMBER(C11), C15&gt;C11), ROUND((D15-D11)/(C15-C11), 2), "")</f>
         <v/>
       </c>
       <c r="J20" s="27" t="inlineStr">
@@ -1162,7 +1153,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21" ht="17" customHeight="1">
       <c r="B21" s="29" t="inlineStr">
         <is>
           <t>Nota: La pendenza di andata è positiva (+), quella di ritorno è negativa (-) perché il verso è opposto.</t>

</xml_diff>

<commit_message>
fix(fisica): aggiorna file excel con punta di inversione a 1,80m e ricalcolo intervalli
</commit_message>
<xml_diff>
--- a/public/fisica/archimede/seconda-elettronica/scheda_laboratorio_A4.xlsx
+++ b/public/fisica/archimede/seconda-elettronica/scheda_laboratorio_A4.xlsx
@@ -898,7 +898,7 @@
     <row r="3" ht="15" customHeight="1">
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Esperienza con rotaia e carrello: studio del moto rettilineo con andata e ritorno (punta 2,30 m)</t>
+          <t>Esperienza con rotaia e carrello: studio del moto rettilineo con andata e ritorno (punta 1,80 m)</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C11" s="10" t="n"/>
       <c r="D11" s="14" t="n">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
@@ -1096,7 +1096,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>Punta di inversione a 2,30 m • Il carrello passa due volte per s = 1,50 m (andata e ritorno).</t>
+          <t>Punta di inversione a 1,80 m • Il carrello passa due volte per s = 1,50 m (andata e ritorno).</t>
         </is>
       </c>
       <c r="C17" s="20" t="n"/>
@@ -1116,7 +1116,7 @@
     <row r="19" ht="17" customHeight="1">
       <c r="B19" s="23" t="inlineStr">
         <is>
-          <t>Pendenza Andata: v_andata = (2,30 m - 0,00 m)/(t_punta - t_0)</t>
+          <t>Pendenza Andata: v_andata = (1,80 m - 0,00 m)/(t_punta - t_0)</t>
         </is>
       </c>
       <c r="E19" s="24">
@@ -1134,7 +1134,7 @@
     <row r="20" ht="17" customHeight="1">
       <c r="B20" s="23" t="inlineStr">
         <is>
-          <t>Pendenza Ritorno: v_ritorno = (0,00 m - 2,30 m)/(t_fine - t_punta)</t>
+          <t>Pendenza Ritorno: v_ritorno = (0,00 m - 1,80 m)/(t_fine - t_punta)</t>
         </is>
       </c>
       <c r="E20" s="26">

</xml_diff>